<commit_message>
Correct 2026-10-26 test rows from patent full text
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Kf9BGN4Y1VnhTqa88N2gbo
</commit_message>
<xml_diff>
--- a/patents/특허_누적.xlsx
+++ b/patents/특허_누적.xlsx
@@ -472,7 +472,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="122">
   <si>
     <t xml:space="preserve">업체 × 설계 분야 누적 건수 (특허목록 시트에서 자동 집계)</t>
   </si>
@@ -618,110 +618,13 @@
     <t xml:space="preserve">2026-01-29</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">냉매</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">칠러</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
+    <t xml:space="preserve">2025-06-17</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">축류단과 원심단을 조합한 냉매 압축기</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">. (</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">원문 미열람</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">제목</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">·</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">검색 요약 기준</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
+    <t xml:space="preserve">냉매(칠러)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[원문확인] 축 한쪽에 축류단→원심단, 반대쪽에 축류단→원심단을 배치한 4단 냉매 압축기(축류+원심 2쌍 배면 배치). 원심단 앞에 축류단을 두어 단당 부하를 나누는 구성.</t>
   </si>
   <si>
     <t xml:space="preserve">https://patents.google.com/patent/WO2026024384A1/en</t>
@@ -733,83 +636,16 @@
     <t xml:space="preserve">US20240247686A1</t>
   </si>
   <si>
-    <t xml:space="preserve">등록</t>
-  </si>
-  <si>
     <t xml:space="preserve">Refrigerant compressor including grooved auxiliary bearing interface</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-04-14</t>
+    <t xml:space="preserve">2024-07-25</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">자기베어링 압축기의 보조</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">백업</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">) </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">베어링 접촉면에 홈을 낸 구조</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">등록번호 미확인</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">.</t>
-    </r>
+    <t xml:space="preserve">2024-01-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[원문확인][참고] 자기베어링으로 축을 띄우는 냉매 압축기에서, 보조(터치다운) 베어링과 축 접촉면에 홈을 낸 구조. 착지 시 마찰·손상 저감 목적. ※이전 '2026-04 등록'은 오류, 2024-07 공개 출원임.</t>
   </si>
   <si>
     <t xml:space="preserve">https://patents.google.com/patent/US20240247686A1/en</t>
@@ -824,130 +660,16 @@
     <t xml:space="preserve">JP2026061434A</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">ターボ圧縮機及び冷凍装置 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">터보 압축기 및 냉동 장치</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
+    <t xml:space="preserve">ターボ圧縮機及び冷凍装置 (터보 압축기 및 냉동 장치)</t>
   </si>
   <si>
     <t xml:space="preserve">2026-04-09</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">터보 압축기</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">·</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">냉동장치</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">내용 미확인이라 분야는 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">'</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">기타</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">'</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">로 둠</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">.</t>
-    </r>
+    <t xml:space="preserve">2024-09-30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[원문확인] 케이싱에 갭센서를 달아 임펠러 날개와 케이싱(슈라우드면) 사이 간극을 측정하고, 제어부가 그 값으로 간극 크기를 제어. 팁 간극 관리로 효율 확보.</t>
   </si>
   <si>
     <t xml:space="preserve">https://patents.google.com/patent/JP2026061434A/en</t>
@@ -957,6 +679,9 @@
   </si>
   <si>
     <t xml:space="preserve">US12584521B2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">등록</t>
   </si>
   <si>
     <r>
@@ -990,23 +715,10 @@
     <t xml:space="preserve">2026-03-24</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">포일 베어링에 능동 댐핑을 추가한 하이브리드 구조</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">.</t>
-    </r>
+    <t xml:space="preserve">2023-07-31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[원문확인] 수동 자기베어링(축·고정부에 내장)으로 반경 방향을 지지하고, 축과 함께 도는 자석이 고정 코일에 유도 전류를 만들어 축 자세 변화를 감지·감쇠하는 하이브리드 베어링. ※에어포일 베어링 아님(이전 분류 오류).</t>
   </si>
   <si>
     <t xml:space="preserve">https://patents.google.com/patent/US12584521B2/en</t>
@@ -1021,40 +733,13 @@
     <t xml:space="preserve">Journal foil air bearing for bidirectional rotation</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">공기</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">블로어</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
+    <t xml:space="preserve">2025-10-30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-04-24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">공기(블로어)</t>
   </si>
   <si>
     <r>
@@ -1065,6 +750,23 @@
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">[</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">원문확인</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">][</t>
     </r>
     <r>
       <rPr>
@@ -1089,6 +791,74 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
+      <t xml:space="preserve">저널 포일 공기 베어링</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">탑포일</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">범프포일 양 끝을 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">'L'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">자로 꺾어 고정부를 만들고 결합 구멍으로 고정</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
       <t xml:space="preserve">정</t>
     </r>
     <r>
@@ -1106,24 +876,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">역 양방향 회전에 쓰는 저널 포일 공기 베어링</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">공개일 미확인</t>
+      <t xml:space="preserve">역 양방향 회전 대응</t>
     </r>
     <r>
       <rPr>
@@ -1136,13 +889,19 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">https://pitchbook.com/profiles/company/482747-05</t>
+    <t xml:space="preserve">https://patents.google.com/patent/WO2025226066A1/en</t>
   </si>
   <si>
     <t xml:space="preserve">US11009043B2</t>
   </si>
   <si>
     <t xml:space="preserve">Turbo compressor including intercooler</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2021-05-18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2017-11-07</t>
   </si>
   <si>
     <r>
@@ -1160,6 +919,23 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
+      <t xml:space="preserve">원문확인</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">][</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
       <t xml:space="preserve">참고</t>
     </r>
     <r>
@@ -1169,7 +945,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">] </t>
+      <t xml:space="preserve">] 1</t>
     </r>
     <r>
       <rPr>
@@ -1177,7 +953,41 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">하우징 안 인터쿨러에서 공기 유로와 수냉 유로가 열교환</t>
+      <t xml:space="preserve">단</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">단 임펠러를 모터 양단에 단 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">단 터보 압축기</t>
     </r>
     <r>
       <rPr>
@@ -1194,7 +1004,92 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">날짜 미확인</t>
+      <t xml:space="preserve">하우징 안에 인터쿨러</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">공기 유로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">냉각 유로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">를 넣어 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">단 압축 공기를 식힌 뒤 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">단으로 보냄</t>
     </r>
     <r>
       <rPr>
@@ -1238,6 +1133,12 @@
     <t xml:space="preserve">Thrust bearing for turbo compressor</t>
   </si>
   <si>
+    <t xml:space="preserve">2021-12-07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2020-03-09</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <sz val="10"/>
@@ -1246,6 +1147,23 @@
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">[</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">원문확인</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">][</t>
     </r>
     <r>
       <rPr>
@@ -1270,7 +1188,24 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">터보 압축기 스러스트 베어링</t>
+      <t xml:space="preserve">스러스트 러너 회전 시 변형이 큰 부위에 맞춰 범프포일</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">탑포일 구조를 바꾼 포일 스러스트 베어링</t>
     </r>
     <r>
       <rPr>
@@ -1287,7 +1222,41 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">날짜 미확인</t>
+      <t xml:space="preserve">유막 두께를 일정하게 유지해 부하 지지력</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">내구성 향상</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. ※</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">분류를 에어포일 베어링으로 수정</t>
     </r>
     <r>
       <rPr>
@@ -1315,31 +1284,7 @@
     <t xml:space="preserve">2024-12-31</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">제어</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">·</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">서지</t>
-    </r>
+    <t xml:space="preserve">2022-03-24</t>
   </si>
   <si>
     <r>
@@ -1357,6 +1302,23 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
+      <t xml:space="preserve">원문확인</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">][</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
       <t xml:space="preserve">참고</t>
     </r>
     <r>
@@ -1366,7 +1328,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">] </t>
+      <t xml:space="preserve">] 1·2 </t>
     </r>
     <r>
       <rPr>
@@ -1374,7 +1336,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">입구 선회를 주는 가변 </t>
+      <t xml:space="preserve">하우징 사이에 가이드 베인 축</t>
     </r>
     <r>
       <rPr>
@@ -1383,7 +1345,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">IGV</t>
+      <t xml:space="preserve">(stem)</t>
     </r>
     <r>
       <rPr>
@@ -1391,7 +1353,41 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">로 운전 범위 확대</t>
+      <t xml:space="preserve">을 끼우고</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">하우징 밖 링기어로 베인 기어를 돌려 각도를 바꾸는 가변 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">IGV. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">축방향 이동 제한 구조 포함</t>
     </r>
     <r>
       <rPr>
@@ -1434,7 +1430,24 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">참고</t>
+      <t xml:space="preserve">원문 미확인 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">- Google </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">일시 차단</t>
     </r>
     <r>
       <rPr>
@@ -1451,7 +1464,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">냉각팬 압력으로 앞쪽 축하중을 상쇄</t>
+      <t xml:space="preserve">냉각팬 압력으로 앞쪽 축하중을 상쇄하는 터보블로어</t>
     </r>
     <r>
       <rPr>
@@ -1460,7 +1473,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">. </t>
+      <t xml:space="preserve">(</t>
     </r>
     <r>
       <rPr>
@@ -1468,7 +1481,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">날짜 미확인</t>
+      <t xml:space="preserve">검색 요약 기준</t>
     </r>
     <r>
       <rPr>
@@ -1477,7 +1490,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">.</t>
+      <t xml:space="preserve">).</t>
     </r>
   </si>
   <si>
@@ -1508,9 +1521,6 @@
     <t xml:space="preserve">상</t>
   </si>
   <si>
-    <t xml:space="preserve">냉매(칠러)</t>
-  </si>
-  <si>
     <t xml:space="preserve">중</t>
   </si>
   <si>
@@ -1518,9 +1528,6 @@
   </si>
   <si>
     <t xml:space="preserve">하</t>
-  </si>
-  <si>
-    <t xml:space="preserve">공기(블로어)</t>
   </si>
   <si>
     <t xml:space="preserve">EP</t>
@@ -2010,6 +2017,12 @@
       <sz val="10"/>
       <name val="WenQuanYi Zen Hei"/>
       <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="WenQuanYi Zen Hei"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -2041,12 +2054,6 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="WenQuanYi Zen Hei"/>
-      <family val="2"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -2210,15 +2217,11 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2227,6 +2230,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2602,11 +2609,11 @@
       </c>
       <c r="D4" s="7" t="n">
         <f aca="false">COUNTIFS(특허목록!$B:$B,$A4,특허목록!$J:$J,D$3)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4" s="7" t="n">
         <f aca="false">COUNTIFS(특허목록!$B:$B,$A4,특허목록!$J:$J,E$3)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F4" s="7" t="n">
         <f aca="false">COUNTIFS(특허목록!$B:$B,$A4,특허목록!$J:$J,F$3)</f>
@@ -2679,11 +2686,11 @@
       </c>
       <c r="J5" s="7" t="n">
         <f aca="false">COUNTIFS(특허목록!$B:$B,$A5,특허목록!$J:$J,J$3)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K5" s="7" t="n">
         <f aca="false">COUNTIFS(특허목록!$B:$B,$A5,특허목록!$J:$J,K$3)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L5" s="8" t="n">
         <f aca="false">SUM(B5:K5)</f>
@@ -2806,7 +2813,7 @@
       </c>
       <c r="B8" s="7" t="n">
         <f aca="false">COUNTIFS(특허목록!$B:$B,$A8,특허목록!$J:$J,B$3)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C8" s="7" t="n">
         <f aca="false">COUNTIFS(특허목록!$B:$B,$A8,특허목록!$J:$J,C$3)</f>
@@ -2842,7 +2849,7 @@
       </c>
       <c r="K8" s="7" t="n">
         <f aca="false">COUNTIFS(특허목록!$B:$B,$A8,특허목록!$J:$J,K$3)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L8" s="8" t="n">
         <f aca="false">SUM(B8:K8)</f>
@@ -2973,11 +2980,11 @@
       </c>
       <c r="D11" s="7" t="n">
         <f aca="false">COUNTIFS(특허목록!$B:$B,$A11,특허목록!$J:$J,D$3)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E11" s="7" t="n">
         <f aca="false">COUNTIFS(특허목록!$B:$B,$A11,특허목록!$J:$J,E$3)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F11" s="7" t="n">
         <f aca="false">COUNTIFS(특허목록!$B:$B,$A11,특허목록!$J:$J,F$3)</f>
@@ -3018,7 +3025,7 @@
       </c>
       <c r="B12" s="11" t="n">
         <f aca="false">SUM(B4:B11)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C12" s="11" t="n">
         <f aca="false">SUM(C4:C11)</f>
@@ -3050,11 +3057,11 @@
       </c>
       <c r="J12" s="11" t="n">
         <f aca="false">SUM(J4:J11)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K12" s="11" t="n">
         <f aca="false">SUM(K4:K11)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L12" s="11" t="n">
         <f aca="false">SUM(L4:L11)</f>
@@ -3172,18 +3179,20 @@
       <c r="H2" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="I2" s="14"/>
+      <c r="I2" s="14" t="s">
+        <v>42</v>
+      </c>
       <c r="J2" s="15" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="K2" s="15" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="L2" s="15" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="M2" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="N2" s="16"/>
       <c r="O2" s="16"/>
@@ -3199,13 +3208,13 @@
         <v>36</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F3" s="15" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G3" s="14" t="s">
         <v>48</v>
@@ -3213,18 +3222,20 @@
       <c r="H3" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="I3" s="14"/>
+      <c r="I3" s="14" t="s">
+        <v>50</v>
+      </c>
       <c r="J3" s="15" t="s">
         <v>5</v>
       </c>
       <c r="K3" s="15" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="L3" s="15" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="M3" s="14" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="N3" s="16"/>
       <c r="O3" s="16"/>
@@ -3237,35 +3248,37 @@
         <v>18</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F4" s="15" t="s">
         <v>39</v>
       </c>
       <c r="G4" s="15" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H4" s="14" t="s">
-        <v>56</v>
-      </c>
-      <c r="I4" s="14"/>
+        <v>57</v>
+      </c>
+      <c r="I4" s="14" t="s">
+        <v>58</v>
+      </c>
       <c r="J4" s="15" t="s">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="K4" s="15" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="L4" s="15" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="M4" s="14" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="N4" s="16"/>
       <c r="O4" s="16"/>
@@ -3278,35 +3291,37 @@
         <v>11</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>47</v>
+        <v>63</v>
       </c>
       <c r="G5" s="14" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="H5" s="14" t="s">
-        <v>62</v>
-      </c>
-      <c r="I5" s="14"/>
+        <v>65</v>
+      </c>
+      <c r="I5" s="14" t="s">
+        <v>66</v>
+      </c>
       <c r="J5" s="15" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K5" s="15" t="s">
         <v>11</v>
       </c>
       <c r="L5" s="15" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="M5" s="14" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="N5" s="16"/>
       <c r="O5" s="16"/>
@@ -3319,33 +3334,37 @@
         <v>19</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="D6" s="14" t="s">
         <v>37</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="F6" s="15" t="s">
         <v>39</v>
       </c>
       <c r="G6" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="H6" s="14"/>
-      <c r="I6" s="14"/>
+        <v>71</v>
+      </c>
+      <c r="H6" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="I6" s="14" t="s">
+        <v>73</v>
+      </c>
       <c r="J6" s="15" t="s">
         <v>4</v>
       </c>
       <c r="K6" s="15" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="L6" s="14" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="M6" s="14" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="N6" s="16"/>
       <c r="O6" s="16"/>
@@ -3358,33 +3377,37 @@
         <v>19</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="F7" s="15" t="s">
-        <v>47</v>
+        <v>63</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>72</v>
-      </c>
-      <c r="H7" s="14"/>
-      <c r="I7" s="14"/>
+        <v>78</v>
+      </c>
+      <c r="H7" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="I7" s="14" t="s">
+        <v>80</v>
+      </c>
       <c r="J7" s="15" t="s">
         <v>8</v>
       </c>
       <c r="K7" s="15" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="L7" s="14" t="s">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="M7" s="14" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="N7" s="16"/>
       <c r="O7" s="16"/>
@@ -3394,36 +3417,40 @@
         <v>35</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="F8" s="15" t="s">
-        <v>47</v>
+        <v>63</v>
       </c>
       <c r="G8" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="H8" s="14"/>
-      <c r="I8" s="14"/>
+        <v>86</v>
+      </c>
+      <c r="H8" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="I8" s="14" t="s">
+        <v>88</v>
+      </c>
       <c r="J8" s="15" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K8" s="15" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="L8" s="14" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="M8" s="14" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="N8" s="16"/>
       <c r="O8" s="16"/>
@@ -3436,35 +3463,37 @@
         <v>16</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="F9" s="15" t="s">
-        <v>47</v>
+        <v>63</v>
       </c>
       <c r="G9" s="14" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="H9" s="14" t="s">
-        <v>84</v>
-      </c>
-      <c r="I9" s="14"/>
+        <v>94</v>
+      </c>
+      <c r="I9" s="14" t="s">
+        <v>95</v>
+      </c>
       <c r="J9" s="15" t="s">
-        <v>85</v>
+        <v>9</v>
       </c>
       <c r="K9" s="15" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="L9" s="14" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="M9" s="14" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="N9" s="16"/>
       <c r="O9" s="16"/>
@@ -3477,19 +3506,19 @@
         <v>20</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="F10" s="15" t="s">
-        <v>47</v>
+        <v>63</v>
       </c>
       <c r="G10" s="15" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="H10" s="14"/>
       <c r="I10" s="14"/>
@@ -3497,13 +3526,13 @@
         <v>6</v>
       </c>
       <c r="K10" s="15" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="L10" s="14" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="M10" s="14" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="N10" s="16"/>
       <c r="O10" s="16"/>
@@ -20405,22 +20434,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="B1" s="18" t="s">
         <v>2</v>
       </c>
       <c r="C1" s="18" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="D1" s="18" t="s">
         <v>39</v>
       </c>
       <c r="E1" s="18" t="s">
-        <v>96</v>
+        <v>43</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -20431,16 +20460,16 @@
         <v>3</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="D2" s="18" t="s">
-        <v>47</v>
+        <v>63</v>
       </c>
       <c r="E2" s="18" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -20451,13 +20480,13 @@
         <v>4</v>
       </c>
       <c r="C3" s="18" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="E3" s="18" t="s">
-        <v>100</v>
+        <v>74</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -20468,7 +20497,7 @@
         <v>5</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>37</v>
@@ -20485,7 +20514,7 @@
         <v>11</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -20496,7 +20525,7 @@
         <v>7</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -20507,7 +20536,7 @@
         <v>8</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -20555,7 +20584,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -20563,17 +20592,17 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="20" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="19" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="19" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -20581,17 +20610,17 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="20" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="19" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="19" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -20605,12 +20634,12 @@
     </row>
     <row r="13" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>